<commit_message>
feat: add SAP ID to student records, result cards, transcripts, and search
</commit_message>
<xml_diff>
--- a/BS_Cyber_Security_All_6_Semesters.xlsx
+++ b/BS_Cyber_Security_All_6_Semesters.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\websites\MyWebsite trans\Generate trnscript\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\websites\Generate trnscript\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C7A366D-107A-4C4C-B746-5F25975513D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47A0B9D6-BF68-44C5-88CA-CCA47B5412CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Semester 1" sheetId="1" r:id="rId1"/>
@@ -22830,7 +22830,7 @@
         <v>3.1</v>
       </c>
       <c r="F60" s="6">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="G60" s="6">
         <v>3.4</v>
@@ -22852,11 +22852,11 @@
       </c>
       <c r="M60" s="6">
         <f t="shared" si="0"/>
-        <v>3.62</v>
+        <v>3.63</v>
       </c>
       <c r="N60" s="6">
         <f t="array" ref="N60">IF(B60="","",ROUND((IFERROR(SUMPRODUCT(INDEX('Semester 1'!$D$7:$I$62,MATCH(B60,'Semester 1'!$B$7:$B$62,0),0),{4,3,3,3,3,0}),0)+IFERROR(SUMPRODUCT(INDEX('Semester 2'!$D$7:$I$64,MATCH(B60,'Semester 2'!$B$7:$B$64,0),0),{4,3,3,3,4,0}),0)+IFERROR(SUMPRODUCT(INDEX('Semester 3'!$D$7:$N$64,MATCH(B60,'Semester 3'!$B$7:$B$64,0),0),{3,1,2,1,2,2,1,2,1,2,2}),0)+IFERROR(SUMPRODUCT(INDEX('Semester 4'!$D$7:$M$64,MATCH(B60,'Semester 4'!$B$7:$B$64,0),0),{2,1,2,1,2,1,2,3,2,2}),0)+IFERROR(SUMPRODUCT(INDEX('Semester 5'!$D$7:$N$54,MATCH(B60,'Semester 5'!$B$7:$B$54,0),0),{2,1,2,1,2,1,2,1,3,2,0}),0)+SUMPRODUCT(D60:L60,{2,1,2,1,2,1,3,3,3}))/105,2))</f>
-        <v>3.53</v>
+        <v>3.54</v>
       </c>
       <c r="O60" s="4" t="str">
         <f t="shared" si="2"/>

</xml_diff>